<commit_message>
Api Project - update
</commit_message>
<xml_diff>
--- a/Day25 - 06.06.2025 - API Project/Task/APIDocs/API-Docs-Response, request format .xlsx
+++ b/Day25 - 06.06.2025 - API Project/Task/APIDocs/API-Docs-Response, request format .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/presidio/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E35C7A-FE97-8845-BC7A-B33C116A226C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{513006B5-E820-DB45-BFB4-48DE179224D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20520" xr2:uid="{DCF091EB-1D05-3943-8393-15F1A1F93415}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="149">
   <si>
     <t>Authentication</t>
   </si>
@@ -944,27 +944,6 @@
     <t>amount = 4000</t>
   </si>
   <si>
-    <t>{
-    "$id": "1",
-    "success": true,
-    "message": "Funds added successfully",
-    "data": {
-        "$id": "2",
-        "id": "0197732c-373d-7753-a385-1d317043fd47",
-        "userId": "6c62f90f-eb84-4dec-b07b-a949d4fd0b11",
-        "balance": 4100,
-        "updatedAt": "2025-06-15T10:41:57.126963Z"
-    },
-    "errors": null
-}</t>
-  </si>
-  <si>
-    <t>Bidders can able to refill the virtaul wallet balance to place the bids</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bidder </t>
-  </si>
-  <si>
     <t>Eagreements</t>
   </si>
   <si>
@@ -1000,6 +979,33 @@
   </si>
   <si>
     <t>User can download their e-agreement from the server</t>
+  </si>
+  <si>
+    <t>api/v1/User/GetWalletHistoryByUserId</t>
+  </si>
+  <si>
+    <t>{
+    "$id": "1",
+    "success": true,
+    "message": "Wallet history retrieved successfully",
+    "data": {
+        "$id": "2",
+        "$values": [
+            {
+                "$id": "3",
+                "id": "019773f9-cfb6-790b-8ff8-b91f4c6baadc",
+                "virtualWalletId": "01976cc9-d837-7326-93d1-7cf3c5dab2e4",
+                "amount": -65500,
+                "description": "Deducted for winning auction 67999d4b-d63d-4389-a19b-5ae4c3b28aa3",
+                "transactionDate": "2025-06-15T14:24:00.947717Z",
+                "virtualWallet": null
+            }]}}</t>
+  </si>
+  <si>
+    <t>Bidder, Admin</t>
+  </si>
+  <si>
+    <t>Users  can able view the transaction history</t>
   </si>
 </sst>
 </file>
@@ -1382,15 +1388,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1408,44 +1405,53 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1805,7 +1811,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0486D23B-FC80-D54F-BC46-49AA6C5157E9}">
-  <dimension ref="A2:T194"/>
+  <dimension ref="A2:T195"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="49.1640625" bestFit="1" customWidth="1"/>
@@ -1819,17 +1825,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -1843,15 +1849,15 @@
       <c r="T2" s="2"/>
     </row>
     <row r="3" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="58"/>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -1865,15 +1871,15 @@
       <c r="T3" s="2"/>
     </row>
     <row r="4" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="59"/>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59"/>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
+      <c r="A4" s="45"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="45"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -2024,39 +2030,39 @@
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A10" s="50" t="s">
+      <c r="A10" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="50"/>
-      <c r="C10" s="50"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="50"/>
-      <c r="G10" s="50"/>
-      <c r="H10" s="50"/>
-      <c r="I10" s="50"/>
+      <c r="B10" s="46"/>
+      <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A11" s="53"/>
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
-      <c r="D11" s="53"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="53"/>
-      <c r="G11" s="53"/>
-      <c r="H11" s="53"/>
-      <c r="I11" s="53"/>
+      <c r="A11" s="47"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A12" s="53"/>
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
-      <c r="D12" s="53"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="53"/>
-      <c r="G12" s="53"/>
-      <c r="H12" s="53"/>
-      <c r="I12" s="53"/>
+      <c r="A12" s="47"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="47"/>
     </row>
     <row r="13" spans="1:20" s="4" customFormat="1" ht="38" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
@@ -2143,7 +2149,7 @@
     </row>
     <row r="16" spans="1:20" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A16" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>35</v>
@@ -2172,7 +2178,7 @@
     </row>
     <row r="17" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A17" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B17" s="13" t="s">
         <v>40</v>
@@ -2201,7 +2207,7 @@
     </row>
     <row r="18" spans="1:9" ht="221" x14ac:dyDescent="0.2">
       <c r="A18" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>125</v>
@@ -2228,41 +2234,41 @@
         <v>111</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="119" x14ac:dyDescent="0.2">
-      <c r="A19" s="35">
-        <v>4</v>
-      </c>
-      <c r="B19" s="39" t="s">
+    <row r="19" spans="1:9" ht="221" x14ac:dyDescent="0.2">
+      <c r="A19" s="7">
+        <v>6</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+      <c r="A20" s="35">
+        <v>7</v>
+      </c>
+      <c r="B20" s="39" t="s">
         <v>44</v>
-      </c>
-      <c r="C19" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="E19" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="F19" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="G19" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="H19" s="39" t="s">
-        <v>48</v>
-      </c>
-      <c r="I19" s="36" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="221" x14ac:dyDescent="0.2">
-      <c r="A20" s="35">
-        <v>5</v>
-      </c>
-      <c r="B20" s="39" t="s">
-        <v>134</v>
       </c>
       <c r="C20" s="36" t="s">
         <v>50</v>
@@ -2271,199 +2277,201 @@
         <v>1</v>
       </c>
       <c r="E20" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="H20" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" s="36" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="306" x14ac:dyDescent="0.2">
+      <c r="A21" s="35">
+        <v>8</v>
+      </c>
+      <c r="B21" s="39" t="s">
+        <v>134</v>
+      </c>
+      <c r="C21" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="37" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" s="38" t="s">
         <v>135</v>
       </c>
-      <c r="F20" s="38" t="s">
+      <c r="F21" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="G20" s="38" t="s">
-        <v>136</v>
-      </c>
-      <c r="H20" s="39" t="s">
-        <v>137</v>
-      </c>
-      <c r="I20" s="36" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A21" s="30">
+      <c r="G21" s="38" t="s">
+        <v>146</v>
+      </c>
+      <c r="H21" s="39" t="s">
+        <v>148</v>
+      </c>
+      <c r="I21" s="36" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A22" s="30">
+        <v>9</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="H22" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="I22" s="32" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+      <c r="A23" s="24">
+        <v>10</v>
+      </c>
+      <c r="B23" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F23" s="24"/>
+      <c r="G23" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="H23" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="I23" s="25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="46"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="46"/>
+      <c r="I24" s="49"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="50"/>
+      <c r="B25" s="47"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="47"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="47"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="51"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="52"/>
+      <c r="B26" s="53"/>
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53"/>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="54"/>
+    </row>
+    <row r="27" spans="1:9" s="4" customFormat="1" ht="44" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="31" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="D21" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="E21" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="F21" s="34" t="s">
-        <v>54</v>
-      </c>
-      <c r="G21" s="34" t="s">
-        <v>55</v>
-      </c>
-      <c r="H21" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="I21" s="32" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="119" x14ac:dyDescent="0.2">
-      <c r="A22" s="24">
+      <c r="G27" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="26" t="b">
-        <v>1</v>
-      </c>
-      <c r="E22" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="F22" s="24"/>
-      <c r="G22" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="H22" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="I22" s="25" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A23" s="49" t="s">
-        <v>63</v>
-      </c>
-      <c r="B23" s="50"/>
-      <c r="C23" s="50"/>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="50"/>
-      <c r="I23" s="51"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A24" s="52"/>
-      <c r="B24" s="53"/>
-      <c r="C24" s="53"/>
-      <c r="D24" s="53"/>
-      <c r="E24" s="53"/>
-      <c r="F24" s="53"/>
-      <c r="G24" s="53"/>
-      <c r="H24" s="53"/>
-      <c r="I24" s="54"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A25" s="55"/>
-      <c r="B25" s="56"/>
-      <c r="C25" s="56"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="57"/>
-    </row>
-    <row r="26" spans="1:9" s="4" customFormat="1" ht="44" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="3" t="s">
+      <c r="H27" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="388" x14ac:dyDescent="0.2">
+      <c r="A28" s="23">
+        <v>1</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="20" t="b">
+        <v>1</v>
+      </c>
+      <c r="E28" s="23"/>
+      <c r="F28" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="G28" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="H28" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="I28" s="19" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="408" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="7">
         <v>2</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="388" x14ac:dyDescent="0.2">
-      <c r="A27" s="23">
-        <v>1</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="E27" s="23"/>
-      <c r="F27" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="G27" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="H27" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="I27" s="19" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="408" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="7">
-        <v>2</v>
-      </c>
-      <c r="B28" s="11" t="s">
+      <c r="B29" s="11" t="s">
         <v>69</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F28" s="7"/>
-      <c r="G28" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="I28" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="114" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="7">
-        <v>3</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>9</v>
@@ -2472,25 +2480,25 @@
         <v>1</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F29" s="7"/>
-      <c r="G29" s="7" t="s">
-        <v>75</v>
+      <c r="G29" s="10" t="s">
+        <v>70</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="I29" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="114" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="7">
-        <v>4</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>77</v>
+        <v>3</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>73</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>9</v>
@@ -2499,25 +2507,25 @@
         <v>1</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F30" s="7"/>
-      <c r="G30" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="H30" s="13" t="s">
-        <v>80</v>
+      <c r="G30" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>76</v>
       </c>
       <c r="I30" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="153" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A31" s="7">
-        <v>5</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>81</v>
+        <v>4</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>77</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>9</v>
@@ -2525,13 +2533,15 @@
       <c r="D31" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="E31" s="7"/>
+      <c r="E31" s="10" t="s">
+        <v>78</v>
+      </c>
       <c r="F31" s="7"/>
       <c r="G31" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="H31" s="11" t="s">
-        <v>83</v>
+        <v>79</v>
+      </c>
+      <c r="H31" s="13" t="s">
+        <v>80</v>
       </c>
       <c r="I31" s="11" t="s">
         <v>49</v>
@@ -2539,10 +2549,10 @@
     </row>
     <row r="32" spans="1:9" ht="153" x14ac:dyDescent="0.2">
       <c r="A32" s="7">
-        <v>6</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>84</v>
+        <v>5</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>81</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>9</v>
@@ -2553,21 +2563,21 @@
       <c r="E32" s="7"/>
       <c r="F32" s="7"/>
       <c r="G32" s="10" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="I32" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="153" x14ac:dyDescent="0.2">
       <c r="A33" s="7">
-        <v>7</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>87</v>
+        <v>6</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>84</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>9</v>
@@ -2575,84 +2585,82 @@
       <c r="D33" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="E33" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="F33" s="10" t="s">
-        <v>88</v>
-      </c>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
       <c r="G33" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="I33" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="30">
+    <row r="34" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+      <c r="A34" s="7">
+        <v>7</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="G34" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="409" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="30">
         <v>8</v>
       </c>
-      <c r="B34" s="32" t="s">
+      <c r="B35" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="C34" s="32" t="s">
+      <c r="C35" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="D34" s="33" t="b">
-        <v>1</v>
-      </c>
-      <c r="E34" s="34" t="s">
+      <c r="D35" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="E35" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="F34" s="34" t="s">
+      <c r="F35" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="G34" s="34" t="s">
+      <c r="G35" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="H34" s="32" t="s">
+      <c r="H35" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="I34" s="32" t="s">
+      <c r="I35" s="32" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A35" s="35">
+    <row r="36" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A36" s="35">
         <v>9</v>
       </c>
-      <c r="B35" s="36" t="s">
+      <c r="B36" s="36" t="s">
         <v>97</v>
-      </c>
-      <c r="C35" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="D35" s="37" t="b">
-        <v>1</v>
-      </c>
-      <c r="E35" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="F35" s="35"/>
-      <c r="G35" s="38" t="s">
-        <v>99</v>
-      </c>
-      <c r="H35" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="I35" s="36" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="238" x14ac:dyDescent="0.2">
-      <c r="A36" s="35">
-        <v>10</v>
-      </c>
-      <c r="B36" s="36" t="s">
-        <v>102</v>
       </c>
       <c r="C36" s="36" t="s">
         <v>50</v>
@@ -2660,171 +2668,171 @@
       <c r="D36" s="37" t="b">
         <v>1</v>
       </c>
-      <c r="E36" s="35"/>
-      <c r="F36" s="38" t="s">
-        <v>103</v>
-      </c>
+      <c r="E36" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="F36" s="35"/>
       <c r="G36" s="38" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="H36" s="39" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="I36" s="36" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="187" x14ac:dyDescent="0.2">
-      <c r="A37" s="24">
+    <row r="37" spans="1:9" ht="238" x14ac:dyDescent="0.2">
+      <c r="A37" s="35">
+        <v>10</v>
+      </c>
+      <c r="B37" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D37" s="37" t="b">
+        <v>1</v>
+      </c>
+      <c r="E37" s="35"/>
+      <c r="F37" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="G37" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="H37" s="39" t="s">
+        <v>105</v>
+      </c>
+      <c r="I37" s="36" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="187" x14ac:dyDescent="0.2">
+      <c r="A38" s="24">
         <v>11</v>
       </c>
-      <c r="B37" s="28" t="s">
+      <c r="B38" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="C37" s="25" t="s">
+      <c r="C38" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="D37" s="26" t="b">
-        <v>1</v>
-      </c>
-      <c r="E37" s="24" t="s">
+      <c r="D38" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E38" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="F37" s="24"/>
-      <c r="G37" s="27" t="s">
+      <c r="F38" s="24"/>
+      <c r="G38" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="H37" s="29" t="s">
+      <c r="H38" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="I37" s="25" t="s">
+      <c r="I38" s="25" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A38" s="47" t="s">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" s="55" t="s">
         <v>106</v>
       </c>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="47"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="47"/>
-      <c r="H38" s="47"/>
-      <c r="I38" s="47"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A39" s="48"/>
-      <c r="B39" s="48"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="48"/>
-      <c r="H39" s="48"/>
-      <c r="I39" s="48"/>
+      <c r="B39" s="55"/>
+      <c r="C39" s="55"/>
+      <c r="D39" s="55"/>
+      <c r="E39" s="55"/>
+      <c r="F39" s="55"/>
+      <c r="G39" s="55"/>
+      <c r="H39" s="55"/>
+      <c r="I39" s="55"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A40" s="48"/>
-      <c r="B40" s="48"/>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="48"/>
-      <c r="H40" s="48"/>
-      <c r="I40" s="48"/>
-    </row>
-    <row r="41" spans="1:9" s="6" customFormat="1" ht="53" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B41" s="5" t="s">
+      <c r="A40" s="56"/>
+      <c r="B40" s="56"/>
+      <c r="C40" s="56"/>
+      <c r="D40" s="56"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="56"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="56"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A41" s="56"/>
+      <c r="B41" s="56"/>
+      <c r="C41" s="56"/>
+      <c r="D41" s="56"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="56"/>
+      <c r="G41" s="56"/>
+      <c r="H41" s="56"/>
+      <c r="I41" s="56"/>
+    </row>
+    <row r="42" spans="1:9" s="6" customFormat="1" ht="53" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C42" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F42" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G41" s="5" t="s">
+      <c r="G42" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H41" s="5" t="s">
+      <c r="H42" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I41" s="5" t="s">
+      <c r="I42" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="140" x14ac:dyDescent="0.2">
-      <c r="A42" s="23">
-        <v>1</v>
-      </c>
-      <c r="B42" s="19" t="s">
+    <row r="43" spans="1:9" ht="140" x14ac:dyDescent="0.2">
+      <c r="A43" s="23">
+        <v>1</v>
+      </c>
+      <c r="B43" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="C42" s="19" t="s">
+      <c r="C43" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="D42" s="20" t="b">
-        <v>1</v>
-      </c>
-      <c r="E42" s="23"/>
-      <c r="F42" s="21" t="s">
+      <c r="D43" s="20" t="b">
+        <v>1</v>
+      </c>
+      <c r="E43" s="23"/>
+      <c r="F43" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="G42" s="21" t="s">
+      <c r="G43" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="18" t="s">
+      <c r="H43" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="I42" s="19" t="s">
+      <c r="I43" s="19" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="170" x14ac:dyDescent="0.2">
-      <c r="A43" s="7">
+    <row r="44" spans="1:9" ht="170" x14ac:dyDescent="0.2">
+      <c r="A44" s="7">
         <v>2</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B44" s="11" t="s">
         <v>112</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D43" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F43" s="7"/>
-      <c r="G43" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="H43" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="I43" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="255" x14ac:dyDescent="0.2">
-      <c r="A44" s="7">
-        <v>3</v>
-      </c>
-      <c r="B44" s="11" t="s">
-        <v>115</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>9</v>
@@ -2833,150 +2841,177 @@
         <v>1</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>116</v>
+        <v>71</v>
       </c>
       <c r="F44" s="7"/>
       <c r="G44" s="10" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="I44" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="119" x14ac:dyDescent="0.2">
-      <c r="A45" s="24">
+    <row r="45" spans="1:9" ht="255" x14ac:dyDescent="0.2">
+      <c r="A45" s="7">
+        <v>3</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="F45" s="7"/>
+      <c r="G45" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="H45" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="I45" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+      <c r="A46" s="24">
         <v>4</v>
       </c>
-      <c r="B45" s="25" t="s">
+      <c r="B46" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="C45" s="25" t="s">
+      <c r="C46" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="D45" s="26" t="b">
-        <v>1</v>
-      </c>
-      <c r="E45" s="24" t="s">
+      <c r="D46" s="26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E46" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="F45" s="24"/>
-      <c r="G45" s="27" t="s">
+      <c r="F46" s="24"/>
+      <c r="G46" s="27" t="s">
         <v>122</v>
       </c>
-      <c r="H45" s="25" t="s">
+      <c r="H46" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="I45" s="25" t="s">
+      <c r="I46" s="25" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" s="42" t="s">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A47" s="57" t="s">
+        <v>136</v>
+      </c>
+      <c r="B47" s="58"/>
+      <c r="C47" s="58"/>
+      <c r="D47" s="58"/>
+      <c r="E47" s="58"/>
+      <c r="F47" s="58"/>
+      <c r="G47" s="58"/>
+      <c r="H47" s="58"/>
+      <c r="I47" s="58"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A48" s="59"/>
+      <c r="B48" s="59"/>
+      <c r="C48" s="59"/>
+      <c r="D48" s="59"/>
+      <c r="E48" s="59"/>
+      <c r="F48" s="59"/>
+      <c r="G48" s="59"/>
+      <c r="H48" s="59"/>
+      <c r="I48" s="59"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" s="59"/>
+      <c r="B49" s="59"/>
+      <c r="C49" s="59"/>
+      <c r="D49" s="59"/>
+      <c r="E49" s="59"/>
+      <c r="F49" s="59"/>
+      <c r="G49" s="59"/>
+      <c r="H49" s="59"/>
+      <c r="I49" s="59"/>
+    </row>
+    <row r="50" spans="1:9" ht="200" x14ac:dyDescent="0.2">
+      <c r="A50" s="40">
+        <v>1</v>
+      </c>
+      <c r="B50" s="40" t="s">
+        <v>137</v>
+      </c>
+      <c r="C50" s="40" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" s="41" t="b">
+        <v>1</v>
+      </c>
+      <c r="E50" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="F50" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="B46" s="40"/>
-      <c r="C46" s="40"/>
-      <c r="D46" s="40"/>
-      <c r="E46" s="40"/>
-      <c r="F46" s="40"/>
-      <c r="G46" s="40"/>
-      <c r="H46" s="40"/>
-      <c r="I46" s="40"/>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" s="41"/>
-      <c r="B47" s="41"/>
-      <c r="C47" s="41"/>
-      <c r="D47" s="41"/>
-      <c r="E47" s="41"/>
-      <c r="F47" s="41"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="41"/>
-      <c r="I47" s="41"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A48" s="41"/>
-      <c r="B48" s="41"/>
-      <c r="C48" s="41"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="41"/>
-      <c r="I48" s="41"/>
-    </row>
-    <row r="49" spans="1:9" ht="200" x14ac:dyDescent="0.2">
-      <c r="A49" s="43">
-        <v>1</v>
-      </c>
-      <c r="B49" s="43" t="s">
+      <c r="H50" s="40" t="s">
         <v>140</v>
       </c>
-      <c r="C49" s="43" t="s">
+      <c r="I50" s="40" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="60" x14ac:dyDescent="0.2">
+      <c r="A51" s="40">
+        <v>2</v>
+      </c>
+      <c r="B51" s="42" t="s">
+        <v>141</v>
+      </c>
+      <c r="C51" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="D49" s="44" t="b">
-        <v>1</v>
-      </c>
-      <c r="E49" s="43" t="s">
-        <v>141</v>
-      </c>
-      <c r="F49" s="43" t="s">
-        <v>26</v>
-      </c>
-      <c r="G49" s="46" t="s">
+      <c r="D51" s="41" t="b">
+        <v>1</v>
+      </c>
+      <c r="E51" s="42" t="s">
         <v>142</v>
       </c>
-      <c r="H49" s="43" t="s">
+      <c r="F51" s="40"/>
+      <c r="G51" s="40" t="s">
         <v>143</v>
       </c>
-      <c r="I49" s="43" t="s">
+      <c r="H51" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="I51" s="40" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="60" x14ac:dyDescent="0.2">
-      <c r="A50" s="43">
-        <v>2</v>
-      </c>
-      <c r="B50" s="45" t="s">
-        <v>144</v>
-      </c>
-      <c r="C50" s="43" t="s">
-        <v>9</v>
-      </c>
-      <c r="D50" s="44" t="b">
-        <v>1</v>
-      </c>
-      <c r="E50" s="45" t="s">
-        <v>145</v>
-      </c>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="H50" s="43" t="s">
-        <v>147</v>
-      </c>
-      <c r="I50" s="43" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
-      <c r="F51" s="1"/>
-      <c r="G51" s="1"/>
-      <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
-    </row>
-    <row r="194" spans="10:10" x14ac:dyDescent="0.2">
-      <c r="J194" t="s">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+    </row>
+    <row r="195" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J195" t="s">
         <v>124</v>
       </c>
     </row>
@@ -2984,9 +3019,9 @@
   <mergeCells count="5">
     <mergeCell ref="A2:I4"/>
     <mergeCell ref="A10:I12"/>
-    <mergeCell ref="A23:I25"/>
-    <mergeCell ref="A38:I40"/>
-    <mergeCell ref="A46:I48"/>
+    <mergeCell ref="A24:I26"/>
+    <mergeCell ref="A39:I41"/>
+    <mergeCell ref="A47:I49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>